<commit_message>
bengshop: adresy w eksporcie menu
</commit_message>
<xml_diff>
--- a/docs/bengshop/research/eksport/MENU_PO_PORZADKU.xlsx
+++ b/docs/bengshop/research/eksport/MENU_PO_PORZADKU.xlsx
@@ -554,7 +554,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Majtki-pole-dance/298</t>
+          <t>https://bengshop.pl/Majtki-pole-dance/298</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -581,7 +581,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Szorty-odkrywajace-posladki/296</t>
+          <t>https://bengshop.pl/Szorty-odkrywajace-posladki/296</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -608,7 +608,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Szorty-z-paskami-na-udach/239</t>
+          <t>https://bengshop.pl/Szorty-z-paskami-na-udach/239</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -635,7 +635,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Majtki-z-paskami-na-udach/297</t>
+          <t>https://bengshop.pl/Majtki-z-paskami-na-udach/297</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -662,7 +662,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Majtki-do-pole-dance-z-wysokim-stanem/299</t>
+          <t>https://bengshop.pl/Majtki-do-pole-dance-z-wysokim-stanem/299</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -689,7 +689,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Szorty-z-wysokim-stanem/232</t>
+          <t>https://bengshop.pl/Szorty-z-wysokim-stanem/232</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -716,7 +716,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Szorty-z-marszczeniem-na-pupie/180</t>
+          <t>https://bengshop.pl/Szorty-z-marszczeniem-na-pupie/180</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -743,7 +743,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Szorty-zaslaniajace-posladki/253</t>
+          <t>https://bengshop.pl/Szorty-zaslaniajace-posladki/253</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -797,7 +797,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Topy-na-wiekszy-biust/243</t>
+          <t>https://bengshop.pl/Topy-na-wiekszy-biust/243</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -824,7 +824,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Topy-do-tanca/294</t>
+          <t>https://bengshop.pl/Topy-do-tanca/294</t>
         </is>
       </c>
       <c r="E14" t="n">
@@ -851,7 +851,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Topy-z-odkrytymi-plecami/245</t>
+          <t>https://bengshop.pl/Topy-z-odkrytymi-plecami/245</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -878,7 +878,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Topy-z-dekoltem/290</t>
+          <t>https://bengshop.pl/Topy-z-dekoltem/290</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -1013,7 +1013,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/STROJE-DO-POLE-DANCE-DLA-DZIECI/426</t>
+          <t>https://bengshop.pl/STROJE-DO-POLE-DANCE-DLA-DZIECI/426</t>
         </is>
       </c>
       <c r="E21" t="n">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/OUTLET/428</t>
+          <t>https://bengshop.pl/OUTLET/428</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -1461,7 +1461,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/TORBA-NA-TRENING/401</t>
+          <t>https://bengshop.pl/TORBA-NA-TRENING/401</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -1812,7 +1812,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/NAKOLANNIKI-DO-EXOTIC/415</t>
+          <t>https://bengshop.pl/NAKOLANNIKI-DO-EXOTIC/415</t>
         </is>
       </c>
       <c r="E50" t="n">
@@ -1839,7 +1839,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/SZORTY-DO-EXOTIC/407</t>
+          <t>https://bengshop.pl/SZORTY-DO-EXOTIC/407</t>
         </is>
       </c>
       <c r="E51" t="n">
@@ -1866,7 +1866,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/BODY-DO-EXOTIC/408</t>
+          <t>https://bengshop.pl/BODY-DO-EXOTIC/408</t>
         </is>
       </c>
       <c r="E52" t="n">
@@ -1893,7 +1893,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/SPODNICZKI-DO-EXOTIC/413</t>
+          <t>https://bengshop.pl/SPODNICZKI-DO-EXOTIC/413</t>
         </is>
       </c>
       <c r="E53" t="n">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/TOPY-DO-EXOTIC/406</t>
+          <t>https://bengshop.pl/TOPY-DO-EXOTIC/406</t>
         </is>
       </c>
       <c r="E54" t="n">
@@ -1947,7 +1947,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/ZESTAWY-DO-EXOTIC/412</t>
+          <t>https://bengshop.pl/ZESTAWY-DO-EXOTIC/412</t>
         </is>
       </c>
       <c r="E55" t="n">
@@ -1974,7 +1974,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/MARKI/179</t>
+          <t>https://bengshop.pl/MARKI/179</t>
         </is>
       </c>
       <c r="E56" s="2" t="n">
@@ -2001,7 +2001,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/BENG/82</t>
+          <t>https://bengshop.pl/BENG/82</t>
         </is>
       </c>
       <c r="E57" t="n">
@@ -2055,7 +2055,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/MIAMI/371</t>
+          <t>https://bengshop.pl/MIAMI/371</t>
         </is>
       </c>
       <c r="E59" t="n">
@@ -2082,7 +2082,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Mesh-Me-Up/353</t>
+          <t>https://bengshop.pl/Mesh-Me-Up/353</t>
         </is>
       </c>
       <c r="E60" t="n">
@@ -2109,7 +2109,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Self-Love/266</t>
+          <t>https://bengshop.pl/Self-Love/266</t>
         </is>
       </c>
       <c r="E61" t="n">
@@ -2136,7 +2136,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/BENG-x-FARYNSKA/395</t>
+          <t>https://bengshop.pl/BENG-x-FARYNSKA/395</t>
         </is>
       </c>
       <c r="E62" t="n">
@@ -2163,7 +2163,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/COMFY/438</t>
+          <t>https://bengshop.pl/COMFY/438</t>
         </is>
       </c>
       <c r="E63" t="n">
@@ -2190,7 +2190,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Colours-of-Beng/202</t>
+          <t>https://bengshop.pl/Colours-of-Beng/202</t>
         </is>
       </c>
       <c r="E64" t="n">
@@ -2217,7 +2217,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/DARE-TO-DESIRE/405</t>
+          <t>https://bengshop.pl/DARE-TO-DESIRE/405</t>
         </is>
       </c>
       <c r="E65" t="n">
@@ -2244,7 +2244,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Girls-of-BENG/427</t>
+          <t>https://bengshop.pl/Girls-of-BENG/427</t>
         </is>
       </c>
       <c r="E66" t="n">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Sport/380</t>
+          <t>https://bengshop.pl/Sport/380</t>
         </is>
       </c>
       <c r="E67" t="n">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/LIMITED/400</t>
+          <t>https://bengshop.pl/LIMITED/400</t>
         </is>
       </c>
       <c r="E68" t="n">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/QUEEN/150</t>
+          <t>https://bengshop.pl/QUEEN/150</t>
         </is>
       </c>
       <c r="E70" t="n">
@@ -2406,7 +2406,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/MOVS/185</t>
+          <t>https://bengshop.pl/MOVS/185</t>
         </is>
       </c>
       <c r="E72" t="n">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/STROJE-KAPIELOWE/386</t>
+          <t>https://bengshop.pl/STROJE-KAPIELOWE/386</t>
         </is>
       </c>
       <c r="E76" s="2" t="n">
@@ -2541,7 +2541,7 @@
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/BUTY-NA-ZAMOWIENIE/189</t>
+          <t>https://bengshop.pl/BUTY-NA-ZAMOWIENIE/189</t>
         </is>
       </c>
       <c r="E77" s="2" t="n">
@@ -2568,7 +2568,7 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/NOWA-KOLEKCJA/430</t>
+          <t>https://bengshop.pl/NOWA-KOLEKCJA/430</t>
         </is>
       </c>
       <c r="E78" s="2" t="n">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/TOP-20/284</t>
+          <t>https://bengshop.pl/TOP-20/284</t>
         </is>
       </c>
       <c r="E79" s="2" t="n">
@@ -2728,7 +2728,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/NOWA-KOLEKCJA/430</t>
+          <t>https://bengshop.pl/NOWA-KOLEKCJA/430</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -2836,7 +2836,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Topy-z-odkrytymi-plecami/245</t>
+          <t>https://bengshop.pl/Topy-z-odkrytymi-plecami/245</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -2876,7 +2876,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Topy-klasyczne/255</t>
+          <t>https://bengshop.pl/Topy-klasyczne/255</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -2920,7 +2920,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Topy-z-paskami/291</t>
+          <t>https://bengshop.pl/Topy-z-paskami/291</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -2964,7 +2964,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Topy-siateczkowe/281</t>
+          <t>https://bengshop.pl/Topy-siateczkowe/281</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Topy-na-wiekszy-biust/243</t>
+          <t>https://bengshop.pl/Topy-na-wiekszy-biust/243</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -3048,7 +3048,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Krotkie-topy/288</t>
+          <t>https://bengshop.pl/Krotkie-topy/288</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -3092,7 +3092,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Topy-z-dlugim-rekawem/289</t>
+          <t>https://bengshop.pl/Topy-z-dlugim-rekawem/289</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -3136,7 +3136,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Topy-z-dekoltem/290</t>
+          <t>https://bengshop.pl/Topy-z-dekoltem/290</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -3176,7 +3176,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Topy-do-tanca/294</t>
+          <t>https://bengshop.pl/Topy-do-tanca/294</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -3216,7 +3216,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Topy-sportowe/295</t>
+          <t>https://bengshop.pl/Topy-sportowe/295</t>
         </is>
       </c>
       <c r="E14" t="n">
@@ -3296,7 +3296,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Szorty-z-wysokim-stanem/232</t>
+          <t>https://bengshop.pl/Szorty-z-wysokim-stanem/232</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -3336,7 +3336,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Szorty-z-marszczeniem-na-pupie/180</t>
+          <t>https://bengshop.pl/Szorty-z-marszczeniem-na-pupie/180</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -3376,7 +3376,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Szorty-bez-marszczenia/181</t>
+          <t>https://bengshop.pl/Szorty-bez-marszczenia/181</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -3420,7 +3420,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Szorty-z-siatki/442</t>
+          <t>https://bengshop.pl/Szorty-z-siatki/442</t>
         </is>
       </c>
       <c r="E19" t="n">
@@ -3464,7 +3464,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Szorty-zaslaniajace-posladki/253</t>
+          <t>https://bengshop.pl/Szorty-zaslaniajace-posladki/253</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -3504,7 +3504,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Szorty-z-paskami-na-udach/239</t>
+          <t>https://bengshop.pl/Szorty-z-paskami-na-udach/239</t>
         </is>
       </c>
       <c r="E21" t="n">
@@ -3544,7 +3544,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Szorty-odkrywajace-posladki/296</t>
+          <t>https://bengshop.pl/Szorty-odkrywajace-posladki/296</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -3584,7 +3584,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Szorty-z-niskim-stanem/170</t>
+          <t>https://bengshop.pl/Szorty-z-niskim-stanem/170</t>
         </is>
       </c>
       <c r="E23" t="n">
@@ -3628,7 +3628,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Majtki-z-paskami-na-udach/297</t>
+          <t>https://bengshop.pl/Majtki-z-paskami-na-udach/297</t>
         </is>
       </c>
       <c r="E24" t="n">
@@ -3668,7 +3668,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Majtki-pole-dance/298</t>
+          <t>https://bengshop.pl/Majtki-pole-dance/298</t>
         </is>
       </c>
       <c r="E25" t="n">
@@ -3704,7 +3704,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Majtki-do-pole-dance-z-wysokim-stanem/299</t>
+          <t>https://bengshop.pl/Majtki-do-pole-dance-z-wysokim-stanem/299</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Szorty-welurowe/251</t>
+          <t>https://bengshop.pl/Szorty-welurowe/251</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -3868,7 +3868,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/STROJE-Z-SIATKI/443</t>
+          <t>https://bengshop.pl/STROJE-Z-SIATKI/443</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -4136,7 +4136,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/STROJE-DO-POLE-DANCE-DLA-DZIECI/426</t>
+          <t>https://bengshop.pl/STROJE-DO-POLE-DANCE-DLA-DZIECI/426</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/TOPY-DO-EXOTIC/406</t>
+          <t>https://bengshop.pl/TOPY-DO-EXOTIC/406</t>
         </is>
       </c>
       <c r="E39" t="n">
@@ -4248,7 +4248,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/SZORTY-DO-EXOTIC/407</t>
+          <t>https://bengshop.pl/SZORTY-DO-EXOTIC/407</t>
         </is>
       </c>
       <c r="E40" t="n">
@@ -4288,7 +4288,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/BODY-DO-EXOTIC/408</t>
+          <t>https://bengshop.pl/BODY-DO-EXOTIC/408</t>
         </is>
       </c>
       <c r="E41" t="n">
@@ -4328,7 +4328,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/ODZIEZ-Z-SIATKI/444</t>
+          <t>https://bengshop.pl/ODZIEZ-Z-SIATKI/444</t>
         </is>
       </c>
       <c r="E42" t="n">
@@ -4372,7 +4372,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/ZESTAWY-DO-EXOTIC/412</t>
+          <t>https://bengshop.pl/ZESTAWY-DO-EXOTIC/412</t>
         </is>
       </c>
       <c r="E43" t="n">
@@ -4412,7 +4412,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/NAKOLANNIKI-DO-EXOTIC/415</t>
+          <t>https://bengshop.pl/NAKOLANNIKI-DO-EXOTIC/415</t>
         </is>
       </c>
       <c r="E44" t="n">
@@ -4452,7 +4452,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/SPODNICZKI-DO-EXOTIC/413</t>
+          <t>https://bengshop.pl/SPODNICZKI-DO-EXOTIC/413</t>
         </is>
       </c>
       <c r="E45" t="n">
@@ -4492,7 +4492,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/LONGSLEEVE-DO-EXOTIC/409</t>
+          <t>https://bengshop.pl/LONGSLEEVE-DO-EXOTIC/409</t>
         </is>
       </c>
       <c r="E46" t="n">
@@ -4536,7 +4536,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/LEGGINSY-DO-EXOTIC/410</t>
+          <t>https://bengshop.pl/LEGGINSY-DO-EXOTIC/410</t>
         </is>
       </c>
       <c r="E47" t="n">
@@ -4580,7 +4580,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/T-SHIRTS/414</t>
+          <t>https://bengshop.pl/T-SHIRTS/414</t>
         </is>
       </c>
       <c r="E48" t="n">
@@ -4624,7 +4624,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/GARTERY-DO-EXOTIC/411</t>
+          <t>https://bengshop.pl/GARTERY-DO-EXOTIC/411</t>
         </is>
       </c>
       <c r="E49" t="n">
@@ -4828,7 +4828,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/AKCESORIA-DO-BUTOW-PLEASER/441</t>
+          <t>https://bengshop.pl/AKCESORIA-DO-BUTOW-PLEASER/441</t>
         </is>
       </c>
       <c r="E54" t="n">
@@ -4872,7 +4872,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/OUTLET/428</t>
+          <t>https://bengshop.pl/OUTLET/428</t>
         </is>
       </c>
       <c r="E55" t="n">
@@ -5328,7 +5328,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/NAKOLANNIKI-DO-EXOTIC-Z-GRIPEM/432</t>
+          <t>https://bengshop.pl/NAKOLANNIKI-DO-EXOTIC-Z-GRIPEM/432</t>
         </is>
       </c>
       <c r="E67" t="n">
@@ -5372,7 +5372,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/ZELOWE-NAKOLANNIKI-DO-TANCA/431</t>
+          <t>https://bengshop.pl/ZELOWE-NAKOLANNIKI-DO-TANCA/431</t>
         </is>
       </c>
       <c r="E68" t="n">
@@ -5452,7 +5452,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/TORBA-NA-TRENING/401</t>
+          <t>https://bengshop.pl/TORBA-NA-TRENING/401</t>
         </is>
       </c>
       <c r="E70" t="n">
@@ -5604,7 +5604,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/SZNUROWKI-DO-BUTOW-PLEASER/398</t>
+          <t>https://bengshop.pl/SZNUROWKI-DO-BUTOW-PLEASER/398</t>
         </is>
       </c>
       <c r="E74" t="n">
@@ -5692,7 +5692,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/STROJE-KAPIELOWE/386</t>
+          <t>https://bengshop.pl/STROJE-KAPIELOWE/386</t>
         </is>
       </c>
       <c r="E76" t="n">
@@ -5728,7 +5728,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Topy-kapielowe/389</t>
+          <t>https://bengshop.pl/Topy-kapielowe/389</t>
         </is>
       </c>
       <c r="E77" t="n">
@@ -5747,7 +5747,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/STROJE-KAPIELOWE/386</t>
+          <t>https://bengshop.pl/STROJE-KAPIELOWE/386</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -5772,7 +5772,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Brazyliany-kapielowe/388</t>
+          <t>https://bengshop.pl/Brazyliany-kapielowe/388</t>
         </is>
       </c>
       <c r="E78" t="n">
@@ -5791,7 +5791,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/STROJE-KAPIELOWE/386</t>
+          <t>https://bengshop.pl/STROJE-KAPIELOWE/386</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -5816,7 +5816,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Stroje-kapielowe-body/387</t>
+          <t>https://bengshop.pl/Stroje-kapielowe-body/387</t>
         </is>
       </c>
       <c r="E79" t="n">
@@ -5835,7 +5835,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/STROJE-KAPIELOWE/386</t>
+          <t>https://bengshop.pl/STROJE-KAPIELOWE/386</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -6988,7 +6988,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/MARKI/179</t>
+          <t>https://bengshop.pl/MARKI/179</t>
         </is>
       </c>
       <c r="E107" t="n">
@@ -7024,7 +7024,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/BENG/82</t>
+          <t>https://bengshop.pl/BENG/82</t>
         </is>
       </c>
       <c r="E108" t="n">
@@ -7096,7 +7096,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/COMFY/438</t>
+          <t>https://bengshop.pl/COMFY/438</t>
         </is>
       </c>
       <c r="E110" t="n">
@@ -7132,7 +7132,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Girls-of-BENG/427</t>
+          <t>https://bengshop.pl/Girls-of-BENG/427</t>
         </is>
       </c>
       <c r="E111" t="n">
@@ -7168,7 +7168,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/BENG-x-FARYNSKA/395</t>
+          <t>https://bengshop.pl/BENG-x-FARYNSKA/395</t>
         </is>
       </c>
       <c r="E112" t="n">
@@ -7204,7 +7204,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/DARE-TO-DESIRE/405</t>
+          <t>https://bengshop.pl/DARE-TO-DESIRE/405</t>
         </is>
       </c>
       <c r="E113" t="n">
@@ -7240,7 +7240,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/LIMITED/400</t>
+          <t>https://bengshop.pl/LIMITED/400</t>
         </is>
       </c>
       <c r="E114" t="n">
@@ -7276,7 +7276,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Sport/380</t>
+          <t>https://bengshop.pl/Sport/380</t>
         </is>
       </c>
       <c r="E115" t="n">
@@ -7312,7 +7312,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/MIAMI/371</t>
+          <t>https://bengshop.pl/MIAMI/371</t>
         </is>
       </c>
       <c r="E116" t="n">
@@ -7348,7 +7348,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Mesh-Me-Up/353</t>
+          <t>https://bengshop.pl/Mesh-Me-Up/353</t>
         </is>
       </c>
       <c r="E117" t="n">
@@ -7384,7 +7384,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Colours-of-Beng/202</t>
+          <t>https://bengshop.pl/Colours-of-Beng/202</t>
         </is>
       </c>
       <c r="E118" t="n">
@@ -7420,7 +7420,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Self-Love/266</t>
+          <t>https://bengshop.pl/Self-Love/266</t>
         </is>
       </c>
       <c r="E119" t="n">
@@ -7456,7 +7456,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/QUEEN/150</t>
+          <t>https://bengshop.pl/QUEEN/150</t>
         </is>
       </c>
       <c r="E120" t="n">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/MOVS/185</t>
+          <t>https://bengshop.pl/MOVS/185</t>
         </is>
       </c>
       <c r="E123" t="n">
@@ -7708,7 +7708,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/TOP-20/284</t>
+          <t>https://bengshop.pl/TOP-20/284</t>
         </is>
       </c>
       <c r="E127" t="n">
@@ -7744,7 +7744,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/BUTY-NA-ZAMOWIENIE/189</t>
+          <t>https://bengshop.pl/BUTY-NA-ZAMOWIENIE/189</t>
         </is>
       </c>
       <c r="E128" t="n">
@@ -7816,7 +7816,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Topy-klasyczne/255</t>
+          <t>https://bengshop.pl/Topy-klasyczne/255</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -7841,7 +7841,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Topy-z-paskami/291</t>
+          <t>https://bengshop.pl/Topy-z-paskami/291</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -7866,7 +7866,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Topy-siateczkowe/281</t>
+          <t>https://bengshop.pl/Topy-siateczkowe/281</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -7891,7 +7891,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Krotkie-topy/288</t>
+          <t>https://bengshop.pl/Krotkie-topy/288</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -7916,7 +7916,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Topy-z-dlugim-rekawem/289</t>
+          <t>https://bengshop.pl/Topy-z-dlugim-rekawem/289</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -7941,7 +7941,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Topy-sportowe/295</t>
+          <t>https://bengshop.pl/Topy-sportowe/295</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -7966,7 +7966,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Szorty-bez-marszczenia/181</t>
+          <t>https://bengshop.pl/Szorty-bez-marszczenia/181</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -7991,7 +7991,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Szorty-z-siatki/442</t>
+          <t>https://bengshop.pl/Szorty-z-siatki/442</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -8016,7 +8016,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Szorty-z-niskim-stanem/170</t>
+          <t>https://bengshop.pl/Szorty-z-niskim-stanem/170</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -8041,7 +8041,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Szorty-welurowe/251</t>
+          <t>https://bengshop.pl/Szorty-welurowe/251</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -8091,7 +8091,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/STROJE-Z-SIATKI/443</t>
+          <t>https://bengshop.pl/STROJE-Z-SIATKI/443</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -8141,7 +8141,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/ODZIEZ-Z-SIATKI/444</t>
+          <t>https://bengshop.pl/ODZIEZ-Z-SIATKI/444</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -8166,7 +8166,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/LONGSLEEVE-DO-EXOTIC/409</t>
+          <t>https://bengshop.pl/LONGSLEEVE-DO-EXOTIC/409</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -8191,7 +8191,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/LEGGINSY-DO-EXOTIC/410</t>
+          <t>https://bengshop.pl/LEGGINSY-DO-EXOTIC/410</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -8216,7 +8216,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/T-SHIRTS/414</t>
+          <t>https://bengshop.pl/T-SHIRTS/414</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -8241,7 +8241,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/GARTERY-DO-EXOTIC/411</t>
+          <t>https://bengshop.pl/GARTERY-DO-EXOTIC/411</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -8291,7 +8291,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/AKCESORIA-DO-BUTOW-PLEASER/441</t>
+          <t>https://bengshop.pl/AKCESORIA-DO-BUTOW-PLEASER/441</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -8341,7 +8341,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/NAKOLANNIKI-DO-EXOTIC-Z-GRIPEM/432</t>
+          <t>https://bengshop.pl/NAKOLANNIKI-DO-EXOTIC-Z-GRIPEM/432</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -8366,7 +8366,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/ZELOWE-NAKOLANNIKI-DO-TANCA/431</t>
+          <t>https://bengshop.pl/ZELOWE-NAKOLANNIKI-DO-TANCA/431</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -8416,7 +8416,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/SZNUROWKI-DO-BUTOW-PLEASER/398</t>
+          <t>https://bengshop.pl/SZNUROWKI-DO-BUTOW-PLEASER/398</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -8466,7 +8466,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Topy-kapielowe/389</t>
+          <t>https://bengshop.pl/Topy-kapielowe/389</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -8481,7 +8481,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/STROJE-KAPIELOWE/386</t>
+          <t>https://bengshop.pl/STROJE-KAPIELOWE/386</t>
         </is>
       </c>
       <c r="E28" t="n">
@@ -8491,7 +8491,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Brazyliany-kapielowe/388</t>
+          <t>https://bengshop.pl/Brazyliany-kapielowe/388</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -8506,7 +8506,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/STROJE-KAPIELOWE/386</t>
+          <t>https://bengshop.pl/STROJE-KAPIELOWE/386</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -8516,7 +8516,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Stroje-kapielowe-body/387</t>
+          <t>https://bengshop.pl/Stroje-kapielowe-body/387</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -8531,7 +8531,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/STROJE-KAPIELOWE/386</t>
+          <t>https://bengshop.pl/STROJE-KAPIELOWE/386</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -8941,7 +8941,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Buty/435</t>
+          <t>https://bengshop.pl/Buty/435</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -8966,7 +8966,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Akcesoria/436</t>
+          <t>https://bengshop.pl/Akcesoria/436</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -8991,7 +8991,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/do-200zl/345</t>
+          <t>https://bengshop.pl/do-200zl/345</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -9016,7 +9016,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Buty-Pleaser-na-prezent/348</t>
+          <t>https://bengshop.pl/Buty-Pleaser-na-prezent/348</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -9041,7 +9041,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/Ubrania/434</t>
+          <t>https://bengshop.pl/Ubrania/434</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -9066,7 +9066,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/do-150-zl/421</t>
+          <t>https://bengshop.pl/do-150-zl/421</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -9091,7 +9091,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/W-zestawie-taniej/155</t>
+          <t>https://bengshop.pl/W-zestawie-taniej/155</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -9116,7 +9116,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/do-100-zl/420</t>
+          <t>https://bengshop.pl/do-100-zl/420</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -9141,7 +9141,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/do-100zl/344</t>
+          <t>https://bengshop.pl/do-100zl/344</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -9166,7 +9166,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/do-200-zl/422</t>
+          <t>https://bengshop.pl/do-200-zl/422</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -9191,7 +9191,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/do-300-zl/423</t>
+          <t>https://bengshop.pl/do-300-zl/423</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -9216,7 +9216,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/do-300zl/346</t>
+          <t>https://bengshop.pl/do-300zl/346</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -9241,7 +9241,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/do-400-zl/424</t>
+          <t>https://bengshop.pl/do-400-zl/424</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -9266,7 +9266,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/do-400zl/347</t>
+          <t>https://bengshop.pl/do-400zl/347</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -9291,7 +9291,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>https://bengshop.pl/pl/c/do-50-zl/419</t>
+          <t>https://bengshop.pl/do-50-zl/419</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">

</xml_diff>